<commit_message>
Update capacity constraints to use production times
</commit_message>
<xml_diff>
--- a/outputs/resultats_complets.xlsx
+++ b/outputs/resultats_complets.xlsx
@@ -529,10 +529,10 @@
         <v>423</v>
       </c>
       <c r="G2" t="n">
-        <v>423</v>
+        <v>146.51</v>
       </c>
       <c r="H2" t="n">
-        <v>100</v>
+        <v>34.6</v>
       </c>
       <c r="I2" t="n">
         <v>1</v>
@@ -547,14 +547,14 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>HDG_C</t>
+          <t>HDG_B</t>
         </is>
       </c>
       <c r="M2" t="n">
-        <v>3172.53</v>
+        <v>3142.1</v>
       </c>
       <c r="N2" t="n">
-        <v>1341981</v>
+        <v>460344</v>
       </c>
     </row>
     <row r="3">
@@ -583,10 +583,10 @@
         <v>356</v>
       </c>
       <c r="G3" t="n">
-        <v>356</v>
+        <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="I3" t="n">
         <v>1</v>
@@ -599,16 +599,12 @@
       <c r="K3" t="n">
         <v>12347</v>
       </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>PPGI_B</t>
-        </is>
-      </c>
+      <c r="L3" t="inlineStr"/>
       <c r="M3" t="n">
-        <v>4433.17</v>
+        <v>0</v>
       </c>
       <c r="N3" t="n">
-        <v>1578208</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -871,14 +867,14 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>BACR_A</t>
+          <t>BACR_C</t>
         </is>
       </c>
       <c r="M8" t="n">
-        <v>2777.98</v>
+        <v>3097.21</v>
       </c>
       <c r="N8" t="n">
-        <v>1083412</v>
+        <v>1207914</v>
       </c>
     </row>
     <row r="9">
@@ -907,10 +903,10 @@
         <v>243</v>
       </c>
       <c r="G9" t="n">
-        <v>169.84</v>
+        <v>243</v>
       </c>
       <c r="H9" t="n">
-        <v>69.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="I9" t="n">
         <v>1</v>
@@ -932,7 +928,7 @@
         <v>1554.12</v>
       </c>
       <c r="N9" t="n">
-        <v>263954</v>
+        <v>377651</v>
       </c>
     </row>
     <row r="10">
@@ -1173,10 +1169,10 @@
         <v>414</v>
       </c>
       <c r="G14" t="n">
-        <v>414</v>
+        <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="I14" t="n">
         <v>2</v>
@@ -1189,16 +1185,12 @@
       <c r="K14" t="n">
         <v>11943</v>
       </c>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t>PPGI_B</t>
-        </is>
-      </c>
+      <c r="L14" t="inlineStr"/>
       <c r="M14" t="n">
-        <v>4339.28</v>
+        <v>0</v>
       </c>
       <c r="N14" t="n">
-        <v>1796462</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -1299,14 +1291,14 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>BACR_C</t>
+          <t>BACR_A</t>
         </is>
       </c>
       <c r="M16" t="n">
-        <v>2947.93</v>
+        <v>2658.72</v>
       </c>
       <c r="N16" t="n">
-        <v>359647</v>
+        <v>324363</v>
       </c>
     </row>
     <row r="17">
@@ -1623,14 +1615,14 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>HDG_C</t>
+          <t>HDG_B</t>
         </is>
       </c>
       <c r="M22" t="n">
-        <v>3091.08</v>
+        <v>3062.52</v>
       </c>
       <c r="N22" t="n">
-        <v>896413</v>
+        <v>888130</v>
       </c>
     </row>
     <row r="23">
@@ -1781,14 +1773,14 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>HDG_C</t>
+          <t>HDG_B</t>
         </is>
       </c>
       <c r="M25" t="n">
-        <v>2548.14</v>
+        <v>2518.24</v>
       </c>
       <c r="N25" t="n">
-        <v>203851</v>
+        <v>201459</v>
       </c>
     </row>
     <row r="26">
@@ -2029,10 +2021,10 @@
         <v>87</v>
       </c>
       <c r="G30" t="n">
-        <v>0</v>
+        <v>87</v>
       </c>
       <c r="H30" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="I30" t="n">
         <v>2</v>
@@ -2045,12 +2037,16 @@
       <c r="K30" t="n">
         <v>8749</v>
       </c>
-      <c r="L30" t="inlineStr"/>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>CRC</t>
+        </is>
+      </c>
       <c r="M30" t="n">
-        <v>0</v>
+        <v>1222.99</v>
       </c>
       <c r="N30" t="n">
-        <v>0</v>
+        <v>106400</v>
       </c>
     </row>
     <row r="31">
@@ -2183,10 +2179,10 @@
         <v>565</v>
       </c>
       <c r="G33" t="n">
-        <v>374.87</v>
+        <v>565</v>
       </c>
       <c r="H33" t="n">
-        <v>66.3</v>
+        <v>100</v>
       </c>
       <c r="I33" t="n">
         <v>3</v>
@@ -2208,7 +2204,7 @@
         <v>1925.7</v>
       </c>
       <c r="N33" t="n">
-        <v>721881</v>
+        <v>1088020</v>
       </c>
     </row>
     <row r="34">
@@ -2345,10 +2341,10 @@
         <v>475</v>
       </c>
       <c r="G36" t="n">
-        <v>475</v>
+        <v>0</v>
       </c>
       <c r="H36" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="I36" t="n">
         <v>3</v>
@@ -2361,16 +2357,12 @@
       <c r="K36" t="n">
         <v>6492</v>
       </c>
-      <c r="L36" t="inlineStr">
-        <is>
-          <t>HRC_DEC</t>
-        </is>
-      </c>
+      <c r="L36" t="inlineStr"/>
       <c r="M36" t="n">
-        <v>386.16</v>
+        <v>0</v>
       </c>
       <c r="N36" t="n">
-        <v>183427</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37">
@@ -2579,14 +2571,14 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>HDG_C</t>
+          <t>HDG_B</t>
         </is>
       </c>
       <c r="M40" t="n">
-        <v>3093.57</v>
+        <v>3063.25</v>
       </c>
       <c r="N40" t="n">
-        <v>532093</v>
+        <v>526880</v>
       </c>
     </row>
     <row r="41">
@@ -2615,10 +2607,10 @@
         <v>187</v>
       </c>
       <c r="G41" t="n">
-        <v>187</v>
+        <v>0</v>
       </c>
       <c r="H41" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="I41" t="n">
         <v>3</v>
@@ -2631,16 +2623,12 @@
       <c r="K41" t="n">
         <v>9018</v>
       </c>
-      <c r="L41" t="inlineStr">
-        <is>
-          <t>CRC</t>
-        </is>
-      </c>
+      <c r="L41" t="inlineStr"/>
       <c r="M41" t="n">
-        <v>1834.39</v>
+        <v>0</v>
       </c>
       <c r="N41" t="n">
-        <v>343030</v>
+        <v>0</v>
       </c>
     </row>
     <row r="42">
@@ -2723,10 +2711,10 @@
         <v>115</v>
       </c>
       <c r="G43" t="n">
-        <v>115</v>
+        <v>62.87</v>
       </c>
       <c r="H43" t="n">
-        <v>100</v>
+        <v>54.7</v>
       </c>
       <c r="I43" t="n">
         <v>3</v>
@@ -2748,7 +2736,7 @@
         <v>1884.58</v>
       </c>
       <c r="N43" t="n">
-        <v>216726</v>
+        <v>118478</v>
       </c>
     </row>
     <row r="44">
@@ -2831,10 +2819,10 @@
         <v>77</v>
       </c>
       <c r="G45" t="n">
-        <v>77</v>
+        <v>0</v>
       </c>
       <c r="H45" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="I45" t="n">
         <v>3</v>
@@ -2847,16 +2835,12 @@
       <c r="K45" t="n">
         <v>8804</v>
       </c>
-      <c r="L45" t="inlineStr">
-        <is>
-          <t>CRC</t>
-        </is>
-      </c>
+      <c r="L45" t="inlineStr"/>
       <c r="M45" t="n">
-        <v>1535.38</v>
+        <v>0</v>
       </c>
       <c r="N45" t="n">
-        <v>118225</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46">
@@ -2903,14 +2887,14 @@
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>BACR_C</t>
+          <t>BACR_A</t>
         </is>
       </c>
       <c r="M46" t="n">
-        <v>2793.58</v>
+        <v>2495.49</v>
       </c>
       <c r="N46" t="n">
-        <v>567097</v>
+        <v>506585</v>
       </c>
     </row>
     <row r="47">
@@ -2989,10 +2973,10 @@
         <v>77</v>
       </c>
       <c r="G48" t="n">
-        <v>77</v>
+        <v>0</v>
       </c>
       <c r="H48" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="I48" t="n">
         <v>3</v>
@@ -3005,16 +2989,12 @@
       <c r="K48" t="n">
         <v>9390</v>
       </c>
-      <c r="L48" t="inlineStr">
-        <is>
-          <t>CRC</t>
-        </is>
-      </c>
+      <c r="L48" t="inlineStr"/>
       <c r="M48" t="n">
-        <v>1635.02</v>
+        <v>0</v>
       </c>
       <c r="N48" t="n">
-        <v>125896</v>
+        <v>0</v>
       </c>
     </row>
     <row r="49">
@@ -3061,14 +3041,14 @@
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>HDG_C</t>
+          <t>HDG_B</t>
         </is>
       </c>
       <c r="M49" t="n">
-        <v>2739.54</v>
+        <v>2710.97</v>
       </c>
       <c r="N49" t="n">
-        <v>2029996</v>
+        <v>2008831</v>
       </c>
     </row>
     <row r="50">
@@ -3147,10 +3127,10 @@
         <v>135</v>
       </c>
       <c r="G51" t="n">
-        <v>135</v>
+        <v>0</v>
       </c>
       <c r="H51" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="I51" t="n">
         <v>4</v>
@@ -3163,16 +3143,12 @@
       <c r="K51" t="n">
         <v>6804</v>
       </c>
-      <c r="L51" t="inlineStr">
-        <is>
-          <t>HRC_DEC</t>
-        </is>
-      </c>
+      <c r="L51" t="inlineStr"/>
       <c r="M51" t="n">
-        <v>627.1</v>
+        <v>0</v>
       </c>
       <c r="N51" t="n">
-        <v>84658</v>
+        <v>0</v>
       </c>
     </row>
     <row r="52">
@@ -3683,10 +3659,10 @@
         <v>650</v>
       </c>
       <c r="G61" t="n">
-        <v>650</v>
+        <v>0</v>
       </c>
       <c r="H61" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="I61" t="n">
         <v>1</v>
@@ -3699,16 +3675,12 @@
       <c r="K61" t="n">
         <v>10350</v>
       </c>
-      <c r="L61" t="inlineStr">
-        <is>
-          <t>HDG_C</t>
-        </is>
-      </c>
+      <c r="L61" t="inlineStr"/>
       <c r="M61" t="n">
-        <v>2893.54</v>
+        <v>0</v>
       </c>
       <c r="N61" t="n">
-        <v>1880798</v>
+        <v>0</v>
       </c>
     </row>
     <row r="62">
@@ -3899,10 +3871,10 @@
         <v>720</v>
       </c>
       <c r="G65" t="n">
-        <v>720</v>
+        <v>0</v>
       </c>
       <c r="H65" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="I65" t="n">
         <v>1</v>
@@ -3915,16 +3887,12 @@
       <c r="K65" t="n">
         <v>10580</v>
       </c>
-      <c r="L65" t="inlineStr">
-        <is>
-          <t>HDG_C</t>
-        </is>
-      </c>
+      <c r="L65" t="inlineStr"/>
       <c r="M65" t="n">
-        <v>3044.01</v>
+        <v>0</v>
       </c>
       <c r="N65" t="n">
-        <v>2191687</v>
+        <v>0</v>
       </c>
     </row>
     <row r="66">
@@ -3992,7 +3960,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D57"/>
+  <dimension ref="A1:D59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4032,7 +4000,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>590.84</v>
+        <v>664</v>
       </c>
     </row>
     <row r="3">
@@ -4050,7 +4018,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>2925</v>
+        <v>1278.51</v>
       </c>
     </row>
     <row r="4">
@@ -4068,7 +4036,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1510</v>
+        <v>1154</v>
       </c>
     </row>
     <row r="5">
@@ -4104,7 +4072,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>284</v>
+        <v>371</v>
       </c>
     </row>
     <row r="7">
@@ -4140,7 +4108,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>1211</v>
+        <v>797</v>
       </c>
     </row>
     <row r="9">
@@ -4176,7 +4144,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>1203.87</v>
+        <v>1000.87</v>
       </c>
     </row>
     <row r="11">
@@ -4240,15 +4208,15 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>HRC DEC</t>
+          <t>CRC</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>475</v>
+        <v>1011</v>
       </c>
     </row>
     <row r="15">
@@ -4262,11 +4230,11 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>CRC</t>
+          <t>HDG</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>1011</v>
+        <v>741</v>
       </c>
     </row>
     <row r="16">
@@ -4280,11 +4248,11 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>HDG</t>
+          <t>PPGI</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>741</v>
+        <v>130</v>
       </c>
     </row>
     <row r="17">
@@ -4298,47 +4266,47 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>PPGI</t>
+          <t>BACR</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>PK</t>
+          <t>CRMB</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>BACR</t>
+          <t>CRC</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>132</v>
+        <v>674.11</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>PK</t>
+          <t>CRMB</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>HRC DEC</t>
+          <t>HDG</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>135</v>
+        <v>1297.98</v>
       </c>
     </row>
     <row r="20">
@@ -4352,11 +4320,11 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>CRC</t>
+          <t>PPGI</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>599.84</v>
+        <v>1171.57</v>
       </c>
     </row>
     <row r="21">
@@ -4370,11 +4338,11 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>HDG</t>
+          <t>BACR</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>2969.54</v>
+        <v>395.94</v>
       </c>
     </row>
     <row r="22">
@@ -4384,15 +4352,15 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>PPGI</t>
+          <t>CRC</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>1532.99</v>
+        <v>376.65</v>
       </c>
     </row>
     <row r="23">
@@ -4402,15 +4370,15 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>BACR</t>
+          <t>HDG</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>395.94</v>
+        <v>2243.47</v>
       </c>
     </row>
     <row r="24">
@@ -4424,11 +4392,11 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>CRC</t>
+          <t>PPGI</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>288.32</v>
+        <v>809.14</v>
       </c>
     </row>
     <row r="25">
@@ -4442,11 +4410,11 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>HDG</t>
+          <t>BACR</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>2243.47</v>
+        <v>164.47</v>
       </c>
     </row>
     <row r="26">
@@ -4456,15 +4424,15 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>PPGI</t>
+          <t>CRC</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>1229.44</v>
+        <v>1016.11</v>
       </c>
     </row>
     <row r="27">
@@ -4474,15 +4442,15 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>BACR</t>
+          <t>HDG</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>164.47</v>
+        <v>1268.02</v>
       </c>
     </row>
     <row r="28">
@@ -4496,11 +4464,11 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>CRC</t>
+          <t>PPGI</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>1222.2</v>
+        <v>371.57</v>
       </c>
     </row>
     <row r="29">
@@ -4514,11 +4482,11 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>HDG</t>
+          <t>BACR</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>1268.02</v>
+        <v>206.09</v>
       </c>
     </row>
     <row r="30">
@@ -4528,15 +4496,15 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>PPGI</t>
+          <t>CRC</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>371.57</v>
+        <v>1026.4</v>
       </c>
     </row>
     <row r="31">
@@ -4546,15 +4514,15 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>BACR</t>
+          <t>HDG</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>206.09</v>
+        <v>752.28</v>
       </c>
     </row>
     <row r="32">
@@ -4568,11 +4536,11 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>CRC</t>
+          <t>PPGI</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>1026.4</v>
+        <v>131.98</v>
       </c>
     </row>
     <row r="33">
@@ -4586,47 +4554,47 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>HDG</t>
+          <t>BACR</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>752.28</v>
+        <v>134.01</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>CRMB</t>
+          <t>BAF</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>PPGI</t>
+          <t>CRC</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>131.98</v>
+        <v>694.96</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>CRMB</t>
+          <t>BAF</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>BACR</t>
+          <t>CRC</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>134.01</v>
+        <v>388.3</v>
       </c>
     </row>
     <row r="36">
@@ -4636,15 +4604,15 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>CRC</t>
+          <t>BACR</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>618.39</v>
+        <v>127.69</v>
       </c>
     </row>
     <row r="37">
@@ -4654,15 +4622,15 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>BACR</t>
+          <t>CRC</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>188.59</v>
+        <v>1047.53</v>
       </c>
     </row>
     <row r="38">
@@ -4672,15 +4640,15 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>CRC</t>
+          <t>BACR</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>297.24</v>
+        <v>212.47</v>
       </c>
     </row>
     <row r="39">
@@ -4690,7 +4658,7 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -4698,17 +4666,17 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>1260</v>
+        <v>1058.14</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>BAF</t>
+          <t>SKP</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -4716,7 +4684,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>1058.14</v>
+        <v>701.98</v>
       </c>
     </row>
     <row r="41">
@@ -4726,7 +4694,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -4734,7 +4702,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>624.64</v>
+        <v>392.22</v>
       </c>
     </row>
     <row r="42">
@@ -4744,7 +4712,7 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -4752,7 +4720,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>300.24</v>
+        <v>1058.12</v>
       </c>
     </row>
     <row r="43">
@@ -4762,7 +4730,7 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -4770,25 +4738,25 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>1272.73</v>
+        <v>1068.83</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>SKP</t>
+          <t>LGA</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>CRC</t>
+          <t>HDG</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>1068.83</v>
+        <v>153.34</v>
       </c>
     </row>
     <row r="45">
@@ -4806,7 +4774,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>1580.41</v>
+        <v>1207.81</v>
       </c>
     </row>
     <row r="46">
@@ -4824,7 +4792,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>219.59</v>
+        <v>408.18</v>
       </c>
     </row>
     <row r="47">
@@ -4838,11 +4806,11 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>PPGI</t>
+          <t>HDG</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>1267.47</v>
+        <v>387.25</v>
       </c>
     </row>
     <row r="48">
@@ -4856,11 +4824,11 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>BACR</t>
+          <t>PPGI</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>169.55</v>
+        <v>834.16</v>
       </c>
     </row>
     <row r="49">
@@ -4870,15 +4838,15 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>PPGI</t>
+          <t>BACR</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>383.07</v>
+        <v>41.87</v>
       </c>
     </row>
     <row r="50">
@@ -4892,11 +4860,11 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>BACR</t>
+          <t>HDG</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>212.47</v>
+        <v>180.02</v>
       </c>
     </row>
     <row r="51">
@@ -4906,7 +4874,7 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
@@ -4914,7 +4882,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>136.06</v>
+        <v>383.07</v>
       </c>
     </row>
     <row r="52">
@@ -4928,39 +4896,39 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>BACR</t>
+          <t>HDG</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>138.15</v>
+        <v>775.55</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>LGB</t>
+          <t>LGA</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>HDG</t>
+          <t>PPGI</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>3061.38</v>
+        <v>136.06</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>LGB</t>
+          <t>LGA</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
@@ -4968,7 +4936,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>190.5</v>
+        <v>138.15</v>
       </c>
     </row>
     <row r="55">
@@ -4978,7 +4946,7 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
@@ -4986,7 +4954,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>2312.85</v>
+        <v>1184.78</v>
       </c>
     </row>
     <row r="56">
@@ -4996,7 +4964,7 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
@@ -5004,7 +4972,7 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>1307.24</v>
+        <v>1925.6</v>
       </c>
     </row>
     <row r="57">
@@ -5014,15 +4982,51 @@
         </is>
       </c>
       <c r="B57" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
+          <t>BACR</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>128.98</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>LGB</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>3</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
           <t>HDG</t>
         </is>
       </c>
-      <c r="D57" t="n">
-        <v>775.55</v>
+      <c r="D58" t="n">
+        <v>1127.22</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>LGB</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>3</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>BACR</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>214.61</v>
       </c>
     </row>
   </sheetData>
@@ -5066,7 +5070,7 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>55.3</v>
+        <v>44.6</v>
       </c>
     </row>
     <row r="3">
@@ -5079,7 +5083,7 @@
         <v>2</v>
       </c>
       <c r="C3" t="n">
-        <v>39.5</v>
+        <v>44.8</v>
       </c>
     </row>
     <row r="4">
@@ -5092,7 +5096,7 @@
         <v>3</v>
       </c>
       <c r="C4" t="n">
-        <v>41.6</v>
+        <v>44.3</v>
       </c>
     </row>
     <row r="5">
@@ -5105,7 +5109,7 @@
         <v>4</v>
       </c>
       <c r="C5" t="n">
-        <v>21.9</v>
+        <v>28.2</v>
       </c>
     </row>
     <row r="6">
@@ -5170,7 +5174,7 @@
         <v>1</v>
       </c>
       <c r="C10" t="n">
-        <v>99.59999999999999</v>
+        <v>64.09999999999999</v>
       </c>
     </row>
     <row r="11">
@@ -5183,7 +5187,7 @@
         <v>2</v>
       </c>
       <c r="C11" t="n">
-        <v>82.90000000000001</v>
+        <v>75.90000000000001</v>
       </c>
     </row>
     <row r="12">
@@ -5196,7 +5200,7 @@
         <v>3</v>
       </c>
       <c r="C12" t="n">
-        <v>55.5</v>
+        <v>51.8</v>
       </c>
     </row>
     <row r="13">
@@ -5222,7 +5226,7 @@
         <v>1</v>
       </c>
       <c r="C14" t="n">
-        <v>64</v>
+        <v>55.2</v>
       </c>
     </row>
     <row r="15">
@@ -5235,7 +5239,7 @@
         <v>2</v>
       </c>
       <c r="C15" t="n">
-        <v>23.6</v>
+        <v>41</v>
       </c>
     </row>
     <row r="16">
@@ -5274,7 +5278,7 @@
         <v>1</v>
       </c>
       <c r="C18" t="n">
-        <v>29.7</v>
+        <v>33.4</v>
       </c>
     </row>
     <row r="19">
@@ -5287,7 +5291,7 @@
         <v>2</v>
       </c>
       <c r="C19" t="n">
-        <v>16.7</v>
+        <v>21.8</v>
       </c>
     </row>
     <row r="20">
@@ -5300,7 +5304,7 @@
         <v>3</v>
       </c>
       <c r="C20" t="n">
-        <v>60.6</v>
+        <v>50.4</v>
       </c>
     </row>
     <row r="21">
@@ -5339,7 +5343,7 @@
         <v>2</v>
       </c>
       <c r="C23" t="n">
-        <v>68.40000000000001</v>
+        <v>63.8</v>
       </c>
     </row>
     <row r="24">
@@ -5352,7 +5356,7 @@
         <v>3</v>
       </c>
       <c r="C24" t="n">
-        <v>28.4</v>
+        <v>28.5</v>
       </c>
     </row>
     <row r="25">
@@ -5365,7 +5369,7 @@
         <v>4</v>
       </c>
       <c r="C25" t="n">
-        <v>13.1</v>
+        <v>57.4</v>
       </c>
     </row>
     <row r="26">
@@ -5378,7 +5382,7 @@
         <v>1</v>
       </c>
       <c r="C26" t="n">
-        <v>77.40000000000001</v>
+        <v>37.2</v>
       </c>
     </row>
     <row r="27">
@@ -5391,7 +5395,7 @@
         <v>2</v>
       </c>
       <c r="C27" t="n">
-        <v>77.09999999999999</v>
+        <v>63.5</v>
       </c>
     </row>
     <row r="28">
@@ -5404,7 +5408,7 @@
         <v>3</v>
       </c>
       <c r="C28" t="n">
-        <v>36.3</v>
+        <v>47.3</v>
       </c>
     </row>
     <row r="29">
@@ -5417,7 +5421,7 @@
         <v>4</v>
       </c>
       <c r="C29" t="n">
-        <v>18.5</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -5431,7 +5435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B41"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5449,401 +5453,211 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>dem_CMD_042</t>
+          <t>cap_time_LGA_S1</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4740.09</v>
+        <v>750530.47</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>dem_CMD_028</t>
+          <t>cap_time_BAF_S3</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>4520.03</v>
+        <v>324111.29</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>dem_CMD_014</t>
+          <t>dem_CMD_042</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>4290.63</v>
+        <v>4740.09</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>dem_CMD_064</t>
+          <t>dem_CMD_020</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4238.67</v>
+        <v>4692.71</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>dem_CMD_054</t>
+          <t>dem_CMD_028</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>4211.49</v>
+        <v>4520.03</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>dem_CMD_063</t>
+          <t>dem_CMD_054</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>4056.81</v>
+        <v>4211.49</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>dem_CMD_020</t>
+          <t>dem_CMD_022</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>3064.33</v>
+        <v>3014.09</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>dem_CMD_022</t>
+          <t>dem_CMD_040</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>3062.52</v>
+        <v>3013.11</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>dem_CMD_006</t>
+          <t>dem_CMD_029</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>2839.58</v>
+        <v>2726.29</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>dem_CMD_012</t>
+          <t>dem_CMD_049</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>2811.19</v>
+        <v>2662.55</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>dem_CMD_019</t>
+          <t>dem_CMD_057</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>2806.04</v>
+        <v>2660.49</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>dem_CMD_046</t>
+          <t>dem_CMD_025</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>2793.58</v>
+        <v>2468.49</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>dem_CMD_008</t>
+          <t>hrc_S320</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>2777.98</v>
+        <v>2322.78</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>dem_CMD_029</t>
+          <t>dem_CMD_006</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>2726.29</v>
+        <v>2156.86</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>dem_CMD_035</t>
+          <t>dem_CMD_064</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2718.59</v>
+        <v>1927.57</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>dem_CMD_049</t>
+          <t>dem_CMD_063</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>2710.97</v>
+        <v>1745.71</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>dem_CMD_015</t>
+          <t>dem_CMD_013</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>2703.85</v>
+        <v>1703.37</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>dem_CMD_065</t>
+          <t>dem_CMD_038</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>2695.98</v>
+        <v>1557.96</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>dem_CMD_057</t>
+          <t>no_cadence_PK_S4_HRC_DEC_x_49_HRC_DEC</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>2660.49</v>
+        <v>627.1</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>dem_CMD_066</t>
+          <t>dem_CMD_008</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>2620.06</v>
+        <v>416.58</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>dem_CMD_062</t>
+          <t>no_cadence_PK_S3_HRC_DEC_x_34_HRC_DEC</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>2573.07</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>dem_CMD_061</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
-        <v>2545.74</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>dem_CMD_039</t>
-        </is>
-      </c>
-      <c r="B24" t="n">
-        <v>2544.98</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>dem_CMD_025</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>2518.24</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>dem_CMD_026</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>2479.44</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>dem_CMD_002</t>
-        </is>
-      </c>
-      <c r="B27" t="n">
-        <v>2433.64</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>hrc_S320</t>
-        </is>
-      </c>
-      <c r="B28" t="n">
-        <v>2322.78</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>dem_CMD_013</t>
-        </is>
-      </c>
-      <c r="B29" t="n">
-        <v>1703.37</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>dem_CMD_038</t>
-        </is>
-      </c>
-      <c r="B30" t="n">
-        <v>1557.96</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>hrc_DX51</t>
-        </is>
-      </c>
-      <c r="B31" t="n">
-        <v>1462.68</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>dem_CMD_040</t>
-        </is>
-      </c>
-      <c r="B32" t="n">
-        <v>1443.27</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>dem_CMD_016</t>
-        </is>
-      </c>
-      <c r="B33" t="n">
-        <v>1327.95</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>dem_CMD_037</t>
-        </is>
-      </c>
-      <c r="B34" t="n">
-        <v>1320.95</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>dem_CMD_044</t>
-        </is>
-      </c>
-      <c r="B35" t="n">
-        <v>1270.03</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>dem_CMD_001</t>
-        </is>
-      </c>
-      <c r="B36" t="n">
-        <v>1202.89</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>dem_CMD_024</t>
-        </is>
-      </c>
-      <c r="B37" t="n">
-        <v>808.48</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>dem_CMD_003</t>
-        </is>
-      </c>
-      <c r="B38" t="n">
-        <v>585.24</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>cap_BAF_S3</t>
-        </is>
-      </c>
-      <c r="B39" t="n">
-        <v>355.03</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>cap_LGA_S1</t>
-        </is>
-      </c>
-      <c r="B40" t="n">
-        <v>305.01</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>dem_CMD_017</t>
-        </is>
-      </c>
-      <c r="B41" t="n">
-        <v>100.84</v>
+        <v>386.16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>